<commit_message>
Inclui imagens dos jogos
</commit_message>
<xml_diff>
--- a/database/seeders/data/jogos.xlsx
+++ b/database/seeders/data/jogos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/18d7ca1878445c33/Área de Trabalho/Estudos/ADS/4º Semestre/PI/projeto-integrador/database/seeders/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/18d7ca1878445c33/Área de Trabalho/Estudos/ADS/4º Semestre/projeto-integrador/database/seeders/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{0A99EBBC-5BB9-43D7-A7B1-60E2AAEF9141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F32B8C9-622D-41AF-8E2C-B68586C75D37}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{0A99EBBC-5BB9-43D7-A7B1-60E2AAEF9141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{648CCC2E-E0A5-484F-AC15-ADD3E895ABCD}"/>
   <bookViews>
-    <workbookView xWindow="4710" yWindow="1410" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -211,94 +211,94 @@
     <t>imagem_url</t>
   </si>
   <si>
-    <t>https://i.ibb.co/Td7KpRv/image-2.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/HL5yXsyr/image-3.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/FcFPPC3/image-4.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/4gKMBvR0/image-5.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/9HQvWmXY/image-6.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/k6hJG9PV/image-7.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/BKHkSPH2/image-8.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/dsvB2W5b/image-10.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/ksnFXn6n/image-11.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/N2BpvsVh/image-12.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/5gf5J0cg/image-14.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/8DCmDT8T/image-15.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/7tqJtgcd/image-16.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/1ynn2G8/image-17.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/WvN70KWF/image-18.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/1YHS8n0B/image-19.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/sdQywvRR/image-20.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/hRj0qS8D/image-21.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/3yzmm9fF/image-22.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/bMPdvXnw/image-23.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/S7wNbLDB/image-24.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/yB460339/image-25.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/VcXgcb5f/image-26.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/cXS3fhk3/image-27.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/Kp7dtJpF/image-28.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/VWtDvqwV/image-29.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/9HD1Q712/image-30.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/YFw1zV6t/image-31.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/tMJtvFkg/image-32.png</t>
-  </si>
-  <si>
-    <t>https://i.ibb.co/LzPfVvv4/image-33.png</t>
+    <t>https://ibb.co/mFFQnVR5</t>
+  </si>
+  <si>
+    <t>https://ibb.co/xtSFWgPj</t>
+  </si>
+  <si>
+    <t>https://ibb.co/vC0nyNgj</t>
+  </si>
+  <si>
+    <t>https://ibb.co/ZpfvMLQD</t>
+  </si>
+  <si>
+    <t>https://ibb.co/Mx1QnFPx</t>
+  </si>
+  <si>
+    <t>https://ibb.co/TDntBR5D</t>
+  </si>
+  <si>
+    <t>https://ibb.co/ds7GKTHN</t>
+  </si>
+  <si>
+    <t>https://ibb.co/rGvsSgL5</t>
+  </si>
+  <si>
+    <t>https://ibb.co/KjhZvB47</t>
+  </si>
+  <si>
+    <t>https://ibb.co/j9GcPnKy</t>
+  </si>
+  <si>
+    <t>https://ibb.co/CKHDwqZV</t>
+  </si>
+  <si>
+    <t>https://ibb.co/tTkDfF9T</t>
+  </si>
+  <si>
+    <t>https://ibb.co/b5RFcKDW</t>
+  </si>
+  <si>
+    <t>https://ibb.co/ccyfC6Fr</t>
+  </si>
+  <si>
+    <t>https://ibb.co/Vc2XgYbQ</t>
+  </si>
+  <si>
+    <t>https://ibb.co/PvQgFpmz</t>
+  </si>
+  <si>
+    <t>https://ibb.co/zWt67scc</t>
+  </si>
+  <si>
+    <t>https://ibb.co/SYkV33Z</t>
+  </si>
+  <si>
+    <t>https://ibb.co/sdV8Hc7y</t>
+  </si>
+  <si>
+    <t>https://ibb.co/RpwN2xkD</t>
+  </si>
+  <si>
+    <t>https://ibb.co/dJmm1Y6R</t>
+  </si>
+  <si>
+    <t>https://ibb.co/G358dfbv</t>
+  </si>
+  <si>
+    <t>https://ibb.co/d04ZrkzF</t>
+  </si>
+  <si>
+    <t>https://ibb.co/LhJ3FNq1</t>
+  </si>
+  <si>
+    <t>https://ibb.co/G4Gp78qn</t>
+  </si>
+  <si>
+    <t>https://ibb.co/nq1t4Wdg</t>
+  </si>
+  <si>
+    <t>https://ibb.co/PZ7wmXpC</t>
+  </si>
+  <si>
+    <t>https://ibb.co/4nXngqfb</t>
+  </si>
+  <si>
+    <t>https://ibb.co/rKbr724D</t>
+  </si>
+  <si>
+    <t>https://ibb.co/zV99vRS8</t>
   </si>
 </sst>
 </file>
@@ -377,10 +377,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -697,7 +693,7 @@
         <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -708,7 +704,7 @@
         <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -774,7 +770,7 @@
         <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>92</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -785,7 +781,7 @@
         <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -796,7 +792,7 @@
         <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -807,7 +803,7 @@
         <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -818,7 +814,7 @@
         <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -829,7 +825,7 @@
         <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -840,7 +836,7 @@
         <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -851,7 +847,7 @@
         <v>46</v>
       </c>
       <c r="C16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -862,7 +858,7 @@
         <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -873,7 +869,7 @@
         <v>48</v>
       </c>
       <c r="C18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -884,7 +880,7 @@
         <v>49</v>
       </c>
       <c r="C19" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -895,7 +891,7 @@
         <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -906,7 +902,7 @@
         <v>51</v>
       </c>
       <c r="C21" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -917,7 +913,7 @@
         <v>52</v>
       </c>
       <c r="C22" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -928,7 +924,7 @@
         <v>53</v>
       </c>
       <c r="C23" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -939,7 +935,7 @@
         <v>54</v>
       </c>
       <c r="C24" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -950,7 +946,7 @@
         <v>55</v>
       </c>
       <c r="C25" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -961,7 +957,7 @@
         <v>56</v>
       </c>
       <c r="C26" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -972,7 +968,7 @@
         <v>57</v>
       </c>
       <c r="C27" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -983,7 +979,7 @@
         <v>58</v>
       </c>
       <c r="C28" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -994,7 +990,7 @@
         <v>59</v>
       </c>
       <c r="C29" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1005,7 +1001,7 @@
         <v>60</v>
       </c>
       <c r="C30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1016,7 +1012,7 @@
         <v>61</v>
       </c>
       <c r="C31" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajusta link das imagens dos jogos
</commit_message>
<xml_diff>
--- a/database/seeders/data/jogos.xlsx
+++ b/database/seeders/data/jogos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/18d7ca1878445c33/Área de Trabalho/Estudos/ADS/4º Semestre/projeto-integrador/database/seeders/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{0A99EBBC-5BB9-43D7-A7B1-60E2AAEF9141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{648CCC2E-E0A5-484F-AC15-ADD3E895ABCD}"/>
+  <xr:revisionPtr revIDLastSave="107" documentId="13_ncr:1_{0A99EBBC-5BB9-43D7-A7B1-60E2AAEF9141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B40A2797-221D-40D2-A7C4-E25CAA360FB0}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -211,94 +211,94 @@
     <t>imagem_url</t>
   </si>
   <si>
-    <t>https://ibb.co/mFFQnVR5</t>
-  </si>
-  <si>
-    <t>https://ibb.co/xtSFWgPj</t>
-  </si>
-  <si>
-    <t>https://ibb.co/vC0nyNgj</t>
-  </si>
-  <si>
-    <t>https://ibb.co/ZpfvMLQD</t>
-  </si>
-  <si>
-    <t>https://ibb.co/Mx1QnFPx</t>
-  </si>
-  <si>
-    <t>https://ibb.co/TDntBR5D</t>
-  </si>
-  <si>
-    <t>https://ibb.co/ds7GKTHN</t>
-  </si>
-  <si>
-    <t>https://ibb.co/rGvsSgL5</t>
-  </si>
-  <si>
-    <t>https://ibb.co/KjhZvB47</t>
-  </si>
-  <si>
-    <t>https://ibb.co/j9GcPnKy</t>
-  </si>
-  <si>
-    <t>https://ibb.co/CKHDwqZV</t>
-  </si>
-  <si>
-    <t>https://ibb.co/tTkDfF9T</t>
-  </si>
-  <si>
-    <t>https://ibb.co/b5RFcKDW</t>
-  </si>
-  <si>
-    <t>https://ibb.co/ccyfC6Fr</t>
-  </si>
-  <si>
-    <t>https://ibb.co/Vc2XgYbQ</t>
-  </si>
-  <si>
-    <t>https://ibb.co/PvQgFpmz</t>
-  </si>
-  <si>
-    <t>https://ibb.co/zWt67scc</t>
-  </si>
-  <si>
-    <t>https://ibb.co/SYkV33Z</t>
-  </si>
-  <si>
-    <t>https://ibb.co/sdV8Hc7y</t>
-  </si>
-  <si>
-    <t>https://ibb.co/RpwN2xkD</t>
-  </si>
-  <si>
-    <t>https://ibb.co/dJmm1Y6R</t>
-  </si>
-  <si>
-    <t>https://ibb.co/G358dfbv</t>
-  </si>
-  <si>
-    <t>https://ibb.co/d04ZrkzF</t>
-  </si>
-  <si>
-    <t>https://ibb.co/LhJ3FNq1</t>
-  </si>
-  <si>
-    <t>https://ibb.co/G4Gp78qn</t>
-  </si>
-  <si>
-    <t>https://ibb.co/nq1t4Wdg</t>
-  </si>
-  <si>
-    <t>https://ibb.co/PZ7wmXpC</t>
-  </si>
-  <si>
-    <t>https://ibb.co/4nXngqfb</t>
-  </si>
-  <si>
-    <t>https://ibb.co/rKbr724D</t>
-  </si>
-  <si>
-    <t>https://ibb.co/zV99vRS8</t>
+    <t>https://i.ibb.co/3YYtx9Tm/image-3.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/tTMLg2ks/image-2.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/HL58wc1H/image-4.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/q3DhryHQ/image-5.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/tT2FBVYT/image-6.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/twNDMc5w/image-7.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/tw38CG10/image-8.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/pvwDFNVZ/image-10.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/GfkK4zwW/image-11.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/QvKtJZRY/image-12.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/5gtLDwPg/image-14.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/HTpC5H3F/image-15.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/mCRZX9qc/image-16.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/tT8yqpnx/image-17.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/7d4KjcYN/image-18.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/dsHmLB99/image-19.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/RrXQDDJ/image-20.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/v6j0Yf9Z/image-21.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/bg9F1SMK/image-22.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/CsPPNGvf/image-23.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/NnyJFgH6/image-24.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/TBMykPF6/image-25.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/84dHCYR9/image-26.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/HfR47bjB/image-27.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/bjvDYfwW/image-28.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/mCL6DZsz/image-29.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/W4M4ph3r/image-30.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/zW8vnVGq/image-31.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/1GyyWq9s/image-32.png</t>
+  </si>
+  <si>
+    <t>https://i.ibb.co/wNYsXTbp/image-33.png</t>
   </si>
 </sst>
 </file>
@@ -377,6 +377,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -671,7 +675,7 @@
   <cols>
     <col min="1" max="1" width="45.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="66.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -770,7 +774,7 @@
         <v>39</v>
       </c>
       <c r="C9" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -781,7 +785,7 @@
         <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -792,7 +796,7 @@
         <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -803,7 +807,7 @@
         <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -814,7 +818,7 @@
         <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -825,7 +829,7 @@
         <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -836,7 +840,7 @@
         <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -847,7 +851,7 @@
         <v>46</v>
       </c>
       <c r="C16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -858,7 +862,7 @@
         <v>47</v>
       </c>
       <c r="C17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -869,7 +873,7 @@
         <v>48</v>
       </c>
       <c r="C18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -880,7 +884,7 @@
         <v>49</v>
       </c>
       <c r="C19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -891,7 +895,7 @@
         <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -902,7 +906,7 @@
         <v>51</v>
       </c>
       <c r="C21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -913,7 +917,7 @@
         <v>52</v>
       </c>
       <c r="C22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -924,7 +928,7 @@
         <v>53</v>
       </c>
       <c r="C23" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -935,7 +939,7 @@
         <v>54</v>
       </c>
       <c r="C24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -946,7 +950,7 @@
         <v>55</v>
       </c>
       <c r="C25" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -957,7 +961,7 @@
         <v>56</v>
       </c>
       <c r="C26" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -968,7 +972,7 @@
         <v>57</v>
       </c>
       <c r="C27" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -979,7 +983,7 @@
         <v>58</v>
       </c>
       <c r="C28" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -990,7 +994,7 @@
         <v>59</v>
       </c>
       <c r="C29" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1001,7 +1005,7 @@
         <v>60</v>
       </c>
       <c r="C30" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1012,10 +1016,11 @@
         <v>61</v>
       </c>
       <c r="C31" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>